<commit_message>
feat: add sub-division support to supervisor management, bulk import, profile, and dashboard
</commit_message>
<xml_diff>
--- a/client/public/Supervisor_Import_Template.xlsx
+++ b/client/public/Supervisor_Import_Template.xlsx
@@ -397,12 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
     <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -418,52 +419,115 @@
       <c r="D1" t="str">
         <v>Password</v>
       </c>
+      <c r="E1" t="str">
+        <v>Sub-Division Name</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>EMP002</v>
+        <v>700489</v>
       </c>
       <c r="B2" t="str">
-        <v>Ramesh Kumar</v>
+        <v>Anup Kumar Pandey</v>
       </c>
       <c r="C2" t="str">
-        <v>9876543211</v>
+        <v>8271504574</v>
       </c>
       <c r="D2" t="str">
-        <v>User@123</v>
+        <v>Passw0rd</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Moran</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>EMP003</v>
+        <v>706827</v>
       </c>
       <c r="B3" t="str">
-        <v>Priya Sharma</v>
+        <v>Bhargav Jyoti Guwala</v>
       </c>
       <c r="C3" t="str">
-        <v>9876543212</v>
+        <v>6002562503</v>
       </c>
       <c r="D3" t="str">
-        <v>User@123</v>
+        <v>Passw0rd</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Charaideo</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>EMP004</v>
+        <v>700495</v>
       </c>
       <c r="B4" t="str">
-        <v>Amit Patel</v>
+        <v>Himanshu Chetia</v>
       </c>
       <c r="C4" t="str">
-        <v>9876543213</v>
+        <v>9864972303</v>
       </c>
       <c r="D4" t="str">
-        <v>User@123</v>
+        <v>Passw0rd</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Sivsagar-I&amp;II</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>700506</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Madhab Borgohain</v>
+      </c>
+      <c r="C5" t="str">
+        <v>9864499561</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Passw0rd</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Demow</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>702791</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Moloyraj Boruah</v>
+      </c>
+      <c r="C6" t="str">
+        <v>9101879312</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Passw0rd</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Amguri</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>700534</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Saik Ali</v>
+      </c>
+      <c r="C7" t="str">
+        <v>6003623758</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Passw0rd</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Nazira</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>